<commit_message>
validation data added - notebook06 added - train best models
</commit_message>
<xml_diff>
--- a/data/in/exog/fuel_supply_cost_2020_2025.xlsx
+++ b/data/in/exog/fuel_supply_cost_2020_2025.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Camilo\Dev\maestria-trabajo-integrador\data\in\exog\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F86DBF1-AB17-4358-9F15-EBC8BEEEBB5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EC23B42-AD18-49C3-9068-2BDE4770948E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="167" formatCode="yyyy\-mm\-dd;@"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -56,6 +56,7 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -98,10 +99,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="167" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -404,7 +405,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E2009"/>
+  <dimension ref="A1:E2040"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.85546875" style="3" customWidth="1"/>
@@ -34029,6 +34030,533 @@
         <v>946.61310998980002</v>
       </c>
     </row>
+    <row r="2010" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2010" s="3">
+        <v>45839</v>
+      </c>
+      <c r="B2010">
+        <v>159.86000000000001</v>
+      </c>
+      <c r="C2010">
+        <v>512.74</v>
+      </c>
+      <c r="D2010">
+        <v>435.23</v>
+      </c>
+      <c r="E2010">
+        <v>966.02</v>
+      </c>
+    </row>
+    <row r="2011" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2011" s="3">
+        <v>45840</v>
+      </c>
+      <c r="B2011">
+        <v>159.86000000000001</v>
+      </c>
+      <c r="C2011">
+        <v>514.83000000000004</v>
+      </c>
+      <c r="D2011">
+        <v>431.05</v>
+      </c>
+      <c r="E2011">
+        <v>965.91</v>
+      </c>
+    </row>
+    <row r="2012" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2012" s="3">
+        <v>45841</v>
+      </c>
+      <c r="B2012">
+        <v>159.87</v>
+      </c>
+      <c r="C2012">
+        <v>511.83</v>
+      </c>
+      <c r="D2012">
+        <v>429.23</v>
+      </c>
+      <c r="E2012">
+        <v>965.91</v>
+      </c>
+    </row>
+    <row r="2013" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2013" s="3">
+        <v>45842</v>
+      </c>
+      <c r="B2013">
+        <v>159.88</v>
+      </c>
+      <c r="C2013">
+        <v>514.28</v>
+      </c>
+      <c r="D2013">
+        <v>429.95</v>
+      </c>
+      <c r="E2013">
+        <v>965.91</v>
+      </c>
+    </row>
+    <row r="2014" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2014" s="3">
+        <v>45843</v>
+      </c>
+      <c r="B2014">
+        <v>159.88</v>
+      </c>
+      <c r="C2014">
+        <v>510.66</v>
+      </c>
+      <c r="D2014">
+        <v>424.34</v>
+      </c>
+      <c r="E2014">
+        <v>965.91</v>
+      </c>
+    </row>
+    <row r="2015" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2015" s="3">
+        <v>45844</v>
+      </c>
+      <c r="B2015">
+        <v>159.88</v>
+      </c>
+      <c r="C2015">
+        <v>509.91</v>
+      </c>
+      <c r="D2015">
+        <v>423.7</v>
+      </c>
+      <c r="E2015">
+        <v>965.91</v>
+      </c>
+    </row>
+    <row r="2016" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2016" s="3">
+        <v>45845</v>
+      </c>
+      <c r="B2016">
+        <v>159.88999999999999</v>
+      </c>
+      <c r="C2016">
+        <v>527.91</v>
+      </c>
+      <c r="D2016">
+        <v>429.72</v>
+      </c>
+      <c r="E2016">
+        <v>965.91</v>
+      </c>
+    </row>
+    <row r="2017" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2017" s="3">
+        <v>45846</v>
+      </c>
+      <c r="B2017">
+        <v>159.88999999999999</v>
+      </c>
+      <c r="C2017">
+        <v>512.78</v>
+      </c>
+      <c r="D2017">
+        <v>427.34</v>
+      </c>
+      <c r="E2017">
+        <v>965.86</v>
+      </c>
+    </row>
+    <row r="2018" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2018" s="3">
+        <v>45847</v>
+      </c>
+      <c r="B2018">
+        <v>159.9</v>
+      </c>
+      <c r="C2018">
+        <v>491.24</v>
+      </c>
+      <c r="D2018">
+        <v>430.5</v>
+      </c>
+      <c r="E2018">
+        <v>965.86</v>
+      </c>
+    </row>
+    <row r="2019" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2019" s="3">
+        <v>45848</v>
+      </c>
+      <c r="B2019">
+        <v>159.91</v>
+      </c>
+      <c r="C2019">
+        <v>511.47</v>
+      </c>
+      <c r="D2019">
+        <v>424.42</v>
+      </c>
+      <c r="E2019">
+        <v>965.86</v>
+      </c>
+    </row>
+    <row r="2020" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2020" s="3">
+        <v>45849</v>
+      </c>
+      <c r="B2020">
+        <v>159.91</v>
+      </c>
+      <c r="C2020">
+        <v>511.47</v>
+      </c>
+      <c r="D2020">
+        <v>426.38</v>
+      </c>
+      <c r="E2020">
+        <v>965.86</v>
+      </c>
+    </row>
+    <row r="2021" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2021" s="3">
+        <v>45850</v>
+      </c>
+      <c r="B2021">
+        <v>159.91</v>
+      </c>
+      <c r="C2021">
+        <v>522.42999999999995</v>
+      </c>
+      <c r="D2021">
+        <v>463.51</v>
+      </c>
+      <c r="E2021">
+        <v>965.86</v>
+      </c>
+    </row>
+    <row r="2022" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2022" s="3">
+        <v>45851</v>
+      </c>
+      <c r="B2022">
+        <v>159.91</v>
+      </c>
+      <c r="C2022">
+        <v>515.05999999999995</v>
+      </c>
+      <c r="D2022">
+        <v>429.28</v>
+      </c>
+      <c r="E2022">
+        <v>965.86</v>
+      </c>
+    </row>
+    <row r="2023" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2023" s="3">
+        <v>45852</v>
+      </c>
+      <c r="B2023">
+        <v>159.91999999999999</v>
+      </c>
+      <c r="C2023">
+        <v>511.24</v>
+      </c>
+      <c r="D2023">
+        <v>425.12</v>
+      </c>
+      <c r="E2023">
+        <v>965.86</v>
+      </c>
+    </row>
+    <row r="2024" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2024" s="3">
+        <v>45853</v>
+      </c>
+      <c r="B2024">
+        <v>159.91999999999999</v>
+      </c>
+      <c r="C2024">
+        <v>510.44</v>
+      </c>
+      <c r="D2024">
+        <v>417.18</v>
+      </c>
+      <c r="E2024">
+        <v>965.9</v>
+      </c>
+    </row>
+    <row r="2025" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2025" s="3">
+        <v>45854</v>
+      </c>
+      <c r="B2025">
+        <v>159.86000000000001</v>
+      </c>
+      <c r="C2025">
+        <v>486.94</v>
+      </c>
+      <c r="D2025">
+        <v>420.07</v>
+      </c>
+      <c r="E2025">
+        <v>965.93</v>
+      </c>
+    </row>
+    <row r="2026" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2026" s="3">
+        <v>45855</v>
+      </c>
+      <c r="B2026">
+        <v>159.81</v>
+      </c>
+      <c r="C2026">
+        <v>510.22</v>
+      </c>
+      <c r="D2026">
+        <v>418.9</v>
+      </c>
+      <c r="E2026">
+        <v>965.93</v>
+      </c>
+    </row>
+    <row r="2027" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2027" s="3">
+        <v>45856</v>
+      </c>
+      <c r="B2027">
+        <v>159.77000000000001</v>
+      </c>
+      <c r="C2027">
+        <v>510.63</v>
+      </c>
+      <c r="D2027">
+        <v>420.39</v>
+      </c>
+      <c r="E2027">
+        <v>965.93</v>
+      </c>
+    </row>
+    <row r="2028" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2028" s="3">
+        <v>45857</v>
+      </c>
+      <c r="B2028">
+        <v>159.72999999999999</v>
+      </c>
+      <c r="C2028">
+        <v>510.71</v>
+      </c>
+      <c r="D2028">
+        <v>423.38</v>
+      </c>
+      <c r="E2028">
+        <v>965.93</v>
+      </c>
+    </row>
+    <row r="2029" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2029" s="3">
+        <v>45858</v>
+      </c>
+      <c r="B2029">
+        <v>159.72999999999999</v>
+      </c>
+      <c r="C2029">
+        <v>508.61</v>
+      </c>
+      <c r="D2029">
+        <v>418.35</v>
+      </c>
+      <c r="E2029">
+        <v>965.93</v>
+      </c>
+    </row>
+    <row r="2030" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2030" s="3">
+        <v>45859</v>
+      </c>
+      <c r="B2030">
+        <v>159.68</v>
+      </c>
+      <c r="C2030">
+        <v>497.39</v>
+      </c>
+      <c r="D2030">
+        <v>425.35</v>
+      </c>
+      <c r="E2030">
+        <v>965.96</v>
+      </c>
+    </row>
+    <row r="2031" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2031" s="3">
+        <v>45860</v>
+      </c>
+      <c r="B2031">
+        <v>159.62</v>
+      </c>
+      <c r="C2031">
+        <v>516.26</v>
+      </c>
+      <c r="D2031">
+        <v>420.56</v>
+      </c>
+      <c r="E2031">
+        <v>965.96</v>
+      </c>
+    </row>
+    <row r="2032" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2032" s="3">
+        <v>45861</v>
+      </c>
+      <c r="B2032">
+        <v>159.51</v>
+      </c>
+      <c r="C2032">
+        <v>481.68</v>
+      </c>
+      <c r="D2032">
+        <v>423.97</v>
+      </c>
+      <c r="E2032">
+        <v>950.99</v>
+      </c>
+    </row>
+    <row r="2033" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2033" s="3">
+        <v>45862</v>
+      </c>
+      <c r="B2033">
+        <v>159.41</v>
+      </c>
+      <c r="C2033">
+        <v>512.61</v>
+      </c>
+      <c r="D2033">
+        <v>425.23</v>
+      </c>
+      <c r="E2033">
+        <v>965.96</v>
+      </c>
+    </row>
+    <row r="2034" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2034" s="3">
+        <v>45863</v>
+      </c>
+      <c r="B2034">
+        <v>159.34</v>
+      </c>
+      <c r="C2034">
+        <v>506.57</v>
+      </c>
+      <c r="D2034">
+        <v>423.35</v>
+      </c>
+      <c r="E2034">
+        <v>965.96</v>
+      </c>
+    </row>
+    <row r="2035" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2035" s="3">
+        <v>45864</v>
+      </c>
+      <c r="B2035">
+        <v>159.19999999999999</v>
+      </c>
+      <c r="C2035">
+        <v>517.83000000000004</v>
+      </c>
+      <c r="D2035">
+        <v>421.47</v>
+      </c>
+      <c r="E2035">
+        <v>965.99</v>
+      </c>
+    </row>
+    <row r="2036" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2036" s="3">
+        <v>45865</v>
+      </c>
+      <c r="B2036">
+        <v>159.19999999999999</v>
+      </c>
+      <c r="C2036">
+        <v>498.47</v>
+      </c>
+      <c r="D2036">
+        <v>426.08</v>
+      </c>
+      <c r="E2036">
+        <v>965.99</v>
+      </c>
+    </row>
+    <row r="2037" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2037" s="3">
+        <v>45866</v>
+      </c>
+      <c r="B2037">
+        <v>159.01</v>
+      </c>
+      <c r="C2037">
+        <v>484.29</v>
+      </c>
+      <c r="D2037">
+        <v>423.49</v>
+      </c>
+      <c r="E2037">
+        <v>966.01</v>
+      </c>
+    </row>
+    <row r="2038" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2038" s="3">
+        <v>45867</v>
+      </c>
+      <c r="B2038">
+        <v>158.88999999999999</v>
+      </c>
+      <c r="C2038">
+        <v>478.43</v>
+      </c>
+      <c r="D2038">
+        <v>444.35</v>
+      </c>
+      <c r="E2038">
+        <v>966.01</v>
+      </c>
+    </row>
+    <row r="2039" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2039" s="3">
+        <v>45868</v>
+      </c>
+      <c r="B2039">
+        <v>158.9</v>
+      </c>
+      <c r="C2039">
+        <v>481.14</v>
+      </c>
+      <c r="D2039">
+        <v>424.98</v>
+      </c>
+      <c r="E2039">
+        <v>966.01</v>
+      </c>
+    </row>
+    <row r="2040" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2040" s="3">
+        <v>45869</v>
+      </c>
+      <c r="B2040">
+        <v>158.68</v>
+      </c>
+      <c r="C2040">
+        <v>483.77</v>
+      </c>
+      <c r="D2040">
+        <v>432.52</v>
+      </c>
+      <c r="E2040">
+        <v>966.01</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>